<commit_message>
ingesta: snapshot 2026-07-30 18:45 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-30/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-30/CORDOBA_JUL26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F77DDB72-3CB3-4C83-96EF-D156253C601A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2EA829-CCD3-4ED2-84AF-4CF55AC36E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
+    <workbookView xWindow="3120" yWindow="2205" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
   <sheets>
     <sheet name="ENERO_2026" sheetId="1" r:id="rId1"/>
@@ -7393,7 +7393,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7866,7 +7866,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -8470,7 +8470,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9079,7 +9079,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9689,7 +9689,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -10044,7 +10044,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="29">
                   <c:v>-1</c:v>
@@ -20003,7 +20003,9 @@
       <c r="AF3" s="25">
         <v>0</v>
       </c>
-      <c r="AG3" s="25"/>
+      <c r="AG3" s="25">
+        <v>0</v>
+      </c>
       <c r="AH3" s="25"/>
       <c r="AI3" s="34"/>
       <c r="AJ3" s="36">
@@ -20111,7 +20113,9 @@
       <c r="AF4" s="25">
         <v>0</v>
       </c>
-      <c r="AG4" s="25"/>
+      <c r="AG4" s="25">
+        <v>0</v>
+      </c>
       <c r="AH4" s="25"/>
       <c r="AI4" s="34"/>
       <c r="AJ4" s="36">
@@ -20219,7 +20223,9 @@
       <c r="AF5" s="25">
         <v>0</v>
       </c>
-      <c r="AG5" s="25"/>
+      <c r="AG5" s="25">
+        <v>0</v>
+      </c>
       <c r="AH5" s="25"/>
       <c r="AI5" s="34"/>
       <c r="AJ5" s="36">
@@ -20327,7 +20333,9 @@
       <c r="AF6" s="25">
         <v>0</v>
       </c>
-      <c r="AG6" s="25"/>
+      <c r="AG6" s="25">
+        <v>0</v>
+      </c>
       <c r="AH6" s="25"/>
       <c r="AI6" s="34"/>
       <c r="AJ6" s="36">
@@ -20539,7 +20547,9 @@
       <c r="AF9" s="25">
         <v>0</v>
       </c>
-      <c r="AG9" s="25"/>
+      <c r="AG9" s="25">
+        <v>0</v>
+      </c>
       <c r="AH9" s="25"/>
       <c r="AI9" s="34"/>
       <c r="AJ9" s="36">
@@ -20725,7 +20735,9 @@
       <c r="AF11" s="25">
         <v>0</v>
       </c>
-      <c r="AG11" s="25"/>
+      <c r="AG11" s="25">
+        <v>0</v>
+      </c>
       <c r="AH11" s="25"/>
       <c r="AI11" s="34"/>
       <c r="AJ11" s="36">
@@ -20831,7 +20843,9 @@
       <c r="AF12" s="25">
         <v>0</v>
       </c>
-      <c r="AG12" s="25"/>
+      <c r="AG12" s="25">
+        <v>0</v>
+      </c>
       <c r="AH12" s="25"/>
       <c r="AI12" s="34"/>
       <c r="AJ12" s="36">
@@ -20939,7 +20953,9 @@
       <c r="AF13" s="25">
         <v>0</v>
       </c>
-      <c r="AG13" s="25"/>
+      <c r="AG13" s="25">
+        <v>0</v>
+      </c>
       <c r="AH13" s="25"/>
       <c r="AI13" s="34"/>
       <c r="AJ13" s="36">
@@ -21045,7 +21061,9 @@
       <c r="AF14" s="25">
         <v>0</v>
       </c>
-      <c r="AG14" s="25"/>
+      <c r="AG14" s="25">
+        <v>0</v>
+      </c>
       <c r="AH14" s="25"/>
       <c r="AI14" s="34"/>
       <c r="AJ14" s="36">
@@ -21153,7 +21171,9 @@
       <c r="AF15" s="25">
         <v>0</v>
       </c>
-      <c r="AG15" s="25"/>
+      <c r="AG15" s="25">
+        <v>0</v>
+      </c>
       <c r="AH15" s="25"/>
       <c r="AI15" s="34"/>
       <c r="AJ15" s="36">
@@ -21380,7 +21400,7 @@
       </c>
       <c r="AG19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AH19" s="26">
         <f t="shared" si="1"/>

</xml_diff>